<commit_message>
Docs: 08_mysql, 01_mongodb(기본), 02_mongodb(기본) 완료
</commit_message>
<xml_diff>
--- a/assignment/term3/18회차_실습체크리스트_김윤지.xlsx
+++ b/assignment/term3/18회차_실습체크리스트_김윤지.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jiwab\Desktop\KB 부캠\KB-ITs-Your-Life\assignment\term3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4532873A-3EB3-43BD-9D5E-BFA5985DCEC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3185551-F151-4AB5-AEDB-BB67A4ADF089}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="1056" windowWidth="11280" windowHeight="11520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="1056" windowWidth="13968" windowHeight="11520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -681,15 +681,15 @@
 </file>
 
 <file path=xl/ctrlProps/ctrlProp10.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" lockText="1" noThreeD="1"/>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" checked="Checked" lockText="1" noThreeD="1"/>
 </file>
 
 <file path=xl/ctrlProps/ctrlProp11.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" lockText="1" noThreeD="1"/>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" checked="Checked" lockText="1" noThreeD="1"/>
 </file>
 
 <file path=xl/ctrlProps/ctrlProp12.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" lockText="1" noThreeD="1"/>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" checked="Checked" lockText="1" noThreeD="1"/>
 </file>
 
 <file path=xl/ctrlProps/ctrlProp13.xml><?xml version="1.0" encoding="utf-8"?>
@@ -701,7 +701,7 @@
 </file>
 
 <file path=xl/ctrlProps/ctrlProp15.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" lockText="1" noThreeD="1"/>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" checked="Checked" lockText="1" noThreeD="1"/>
 </file>
 
 <file path=xl/ctrlProps/ctrlProp16.xml><?xml version="1.0" encoding="utf-8"?>
@@ -709,7 +709,7 @@
 </file>
 
 <file path=xl/ctrlProps/ctrlProp17.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" lockText="1" noThreeD="1"/>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" checked="Checked" lockText="1" noThreeD="1"/>
 </file>
 
 <file path=xl/ctrlProps/ctrlProp18.xml><?xml version="1.0" encoding="utf-8"?>
@@ -729,11 +729,11 @@
 </file>
 
 <file path=xl/ctrlProps/ctrlProp21.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" lockText="1" noThreeD="1"/>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" checked="Checked" lockText="1" noThreeD="1"/>
 </file>
 
 <file path=xl/ctrlProps/ctrlProp22.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" lockText="1" noThreeD="1"/>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" checked="Checked" lockText="1" noThreeD="1"/>
 </file>
 
 <file path=xl/ctrlProps/ctrlProp3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -761,7 +761,7 @@
 </file>
 
 <file path=xl/ctrlProps/ctrlProp9.xml><?xml version="1.0" encoding="utf-8"?>
-<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" lockText="1" noThreeD="1"/>
+<formControlPr xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" objectType="CheckBox" checked="Checked" lockText="1" noThreeD="1"/>
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>